<commit_message>
Added Buy & Hold Added Cash Improved Environment files
</commit_message>
<xml_diff>
--- a/Output/Stats.xlsx
+++ b/Output/Stats.xlsx
@@ -453,14 +453,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M28"/>
+  <dimension ref="A1:U28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr"/>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Equal</t>
+          <t>S&amp;P BnH</t>
         </is>
       </c>
       <c r="C1" s="1" t="n"/>
@@ -468,7 +468,7 @@
       <c r="E1" s="1" t="n"/>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Markowitz</t>
+          <t>Equal</t>
         </is>
       </c>
       <c r="G1" s="1" t="n"/>
@@ -476,12 +476,28 @@
       <c r="I1" s="1" t="n"/>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>MAD</t>
+          <t>Markowitz</t>
         </is>
       </c>
       <c r="K1" s="1" t="n"/>
       <c r="L1" s="1" t="n"/>
       <c r="M1" s="1" t="n"/>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>MAD</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="n"/>
+      <c r="P1" s="1" t="n"/>
+      <c r="Q1" s="1" t="n"/>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>MedAD</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="n"/>
+      <c r="T1" s="1" t="n"/>
+      <c r="U1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr"/>
@@ -545,6 +561,46 @@
           <t>Max Drawdown</t>
         </is>
       </c>
+      <c r="N2" s="1" t="inlineStr">
+        <is>
+          <t>Annual Return</t>
+        </is>
+      </c>
+      <c r="O2" s="1" t="inlineStr">
+        <is>
+          <t>Volatility</t>
+        </is>
+      </c>
+      <c r="P2" s="1" t="inlineStr">
+        <is>
+          <t>Sharpe Ratio</t>
+        </is>
+      </c>
+      <c r="Q2" s="1" t="inlineStr">
+        <is>
+          <t>Max Drawdown</t>
+        </is>
+      </c>
+      <c r="R2" s="1" t="inlineStr">
+        <is>
+          <t>Annual Return</t>
+        </is>
+      </c>
+      <c r="S2" s="1" t="inlineStr">
+        <is>
+          <t>Volatility</t>
+        </is>
+      </c>
+      <c r="T2" s="1" t="inlineStr">
+        <is>
+          <t>Sharpe Ratio</t>
+        </is>
+      </c>
+      <c r="U2" s="1" t="inlineStr">
+        <is>
+          <t>Max Drawdown</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -558,40 +614,64 @@
         <v>2000</v>
       </c>
       <c r="B4" t="n">
+        <v>-10.14</v>
+      </c>
+      <c r="C4" t="n">
+        <v>22.22</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-0.4563</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-17.2</v>
+      </c>
+      <c r="F4" t="n">
         <v>1.99</v>
       </c>
-      <c r="C4" t="n">
+      <c r="G4" t="n">
         <v>18.21</v>
       </c>
-      <c r="D4" t="n">
+      <c r="H4" t="n">
         <v>0.1094</v>
       </c>
-      <c r="E4" t="n">
+      <c r="I4" t="n">
         <v>-13.7</v>
       </c>
-      <c r="F4" t="n">
-        <v>-11.84</v>
-      </c>
-      <c r="G4" t="n">
-        <v>21.71</v>
-      </c>
-      <c r="H4" t="n">
-        <v>-0.5456</v>
-      </c>
-      <c r="I4" t="n">
-        <v>-18.44</v>
-      </c>
       <c r="J4" t="n">
-        <v>-11.84</v>
+        <v>4.43</v>
       </c>
       <c r="K4" t="n">
-        <v>21.71</v>
+        <v>11.84</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.5456</v>
+        <v>0.3743</v>
       </c>
       <c r="M4" t="n">
-        <v>-18.44</v>
+        <v>-10.93</v>
+      </c>
+      <c r="N4" t="n">
+        <v>-5.81</v>
+      </c>
+      <c r="O4" t="n">
+        <v>11.12</v>
+      </c>
+      <c r="P4" t="n">
+        <v>-0.5223</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>-9.16</v>
+      </c>
+      <c r="R4" t="n">
+        <v>-41.88</v>
+      </c>
+      <c r="S4" t="n">
+        <v>43.61</v>
+      </c>
+      <c r="T4" t="n">
+        <v>-0.9603</v>
+      </c>
+      <c r="U4" t="n">
+        <v>-52.66</v>
       </c>
     </row>
     <row r="5">
@@ -599,40 +679,64 @@
         <v>2001</v>
       </c>
       <c r="B5" t="n">
+        <v>-13.04</v>
+      </c>
+      <c r="C5" t="n">
+        <v>21.56</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-0.605</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-29.7</v>
+      </c>
+      <c r="F5" t="n">
         <v>-6.44</v>
       </c>
-      <c r="C5" t="n">
+      <c r="G5" t="n">
         <v>19.27</v>
       </c>
-      <c r="D5" t="n">
+      <c r="H5" t="n">
         <v>-0.3344</v>
       </c>
-      <c r="E5" t="n">
+      <c r="I5" t="n">
         <v>-25.27</v>
       </c>
-      <c r="F5" t="n">
-        <v>-11.15</v>
-      </c>
-      <c r="G5" t="n">
-        <v>15.84</v>
-      </c>
-      <c r="H5" t="n">
-        <v>-0.7037</v>
-      </c>
-      <c r="I5" t="n">
-        <v>-19.71</v>
-      </c>
       <c r="J5" t="n">
-        <v>-11.15</v>
+        <v>-6.89</v>
       </c>
       <c r="K5" t="n">
-        <v>15.84</v>
+        <v>8.710000000000001</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.7037</v>
+        <v>-0.7911</v>
       </c>
       <c r="M5" t="n">
-        <v>-19.71</v>
+        <v>-9.59</v>
+      </c>
+      <c r="N5" t="n">
+        <v>-4.48</v>
+      </c>
+      <c r="O5" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="P5" t="n">
+        <v>-0.7012</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>-7.22</v>
+      </c>
+      <c r="R5" t="n">
+        <v>-11.36</v>
+      </c>
+      <c r="S5" t="n">
+        <v>15.61</v>
+      </c>
+      <c r="T5" t="n">
+        <v>-0.7278</v>
+      </c>
+      <c r="U5" t="n">
+        <v>-18.2</v>
       </c>
     </row>
     <row r="6">
@@ -640,40 +744,64 @@
         <v>2002</v>
       </c>
       <c r="B6" t="n">
+        <v>-23.37</v>
+      </c>
+      <c r="C6" t="n">
+        <v>26.03</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-0.8977000000000001</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-33.75</v>
+      </c>
+      <c r="F6" t="n">
         <v>-17.95</v>
       </c>
-      <c r="C6" t="n">
+      <c r="G6" t="n">
         <v>24.63</v>
       </c>
-      <c r="D6" t="n">
+      <c r="H6" t="n">
         <v>-0.7285</v>
       </c>
-      <c r="E6" t="n">
+      <c r="I6" t="n">
         <v>-31.98</v>
       </c>
-      <c r="F6" t="n">
-        <v>-10.74</v>
-      </c>
-      <c r="G6" t="n">
-        <v>24.47</v>
-      </c>
-      <c r="H6" t="n">
-        <v>-0.4388</v>
-      </c>
-      <c r="I6" t="n">
-        <v>-26.35</v>
-      </c>
       <c r="J6" t="n">
-        <v>-10.74</v>
+        <v>-5.72</v>
       </c>
       <c r="K6" t="n">
-        <v>24.47</v>
+        <v>10.72</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.4388</v>
+        <v>-0.5334</v>
       </c>
       <c r="M6" t="n">
-        <v>-26.35</v>
+        <v>-12.52</v>
+      </c>
+      <c r="N6" t="n">
+        <v>-4.57</v>
+      </c>
+      <c r="O6" t="n">
+        <v>9.76</v>
+      </c>
+      <c r="P6" t="n">
+        <v>-0.4686</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>-11.69</v>
+      </c>
+      <c r="R6" t="n">
+        <v>-9.27</v>
+      </c>
+      <c r="S6" t="n">
+        <v>22.31</v>
+      </c>
+      <c r="T6" t="n">
+        <v>-0.4157</v>
+      </c>
+      <c r="U6" t="n">
+        <v>-23.48</v>
       </c>
     </row>
     <row r="7">
@@ -681,40 +809,64 @@
         <v>2003</v>
       </c>
       <c r="B7" t="n">
+        <v>26.38</v>
+      </c>
+      <c r="C7" t="n">
+        <v>17.07</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1.5456</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-14.05</v>
+      </c>
+      <c r="F7" t="n">
         <v>28.57</v>
       </c>
-      <c r="C7" t="n">
+      <c r="G7" t="n">
         <v>15.38</v>
       </c>
-      <c r="D7" t="n">
+      <c r="H7" t="n">
         <v>1.8579</v>
       </c>
-      <c r="E7" t="n">
+      <c r="I7" t="n">
         <v>-13.1</v>
       </c>
-      <c r="F7" t="n">
-        <v>27.3</v>
-      </c>
-      <c r="G7" t="n">
-        <v>15.24</v>
-      </c>
-      <c r="H7" t="n">
-        <v>1.7917</v>
-      </c>
-      <c r="I7" t="n">
-        <v>-12.15</v>
-      </c>
       <c r="J7" t="n">
-        <v>27.3</v>
+        <v>4.97</v>
       </c>
       <c r="K7" t="n">
-        <v>15.24</v>
+        <v>4.01</v>
       </c>
       <c r="L7" t="n">
-        <v>1.7917</v>
+        <v>1.2386</v>
       </c>
       <c r="M7" t="n">
-        <v>-12.15</v>
+        <v>-2.88</v>
+      </c>
+      <c r="N7" t="n">
+        <v>6.74</v>
+      </c>
+      <c r="O7" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="P7" t="n">
+        <v>1.3227</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>-3.82</v>
+      </c>
+      <c r="R7" t="n">
+        <v>18.43</v>
+      </c>
+      <c r="S7" t="n">
+        <v>11.29</v>
+      </c>
+      <c r="T7" t="n">
+        <v>1.6326</v>
+      </c>
+      <c r="U7" t="n">
+        <v>-8.970000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -722,16 +874,16 @@
         <v>2004</v>
       </c>
       <c r="B8" t="n">
-        <v>14.24</v>
+        <v>8.99</v>
       </c>
       <c r="C8" t="n">
-        <v>10.67</v>
+        <v>11.09</v>
       </c>
       <c r="D8" t="n">
-        <v>1.3345</v>
+        <v>0.8107</v>
       </c>
       <c r="E8" t="n">
-        <v>-6</v>
+        <v>-8.16</v>
       </c>
       <c r="F8" t="n">
         <v>14.24</v>
@@ -740,22 +892,46 @@
         <v>10.67</v>
       </c>
       <c r="H8" t="n">
-        <v>1.3342</v>
+        <v>1.3345</v>
       </c>
       <c r="I8" t="n">
         <v>-6</v>
       </c>
       <c r="J8" t="n">
-        <v>14.24</v>
+        <v>12.15</v>
       </c>
       <c r="K8" t="n">
-        <v>10.67</v>
+        <v>7.49</v>
       </c>
       <c r="L8" t="n">
-        <v>1.3342</v>
+        <v>1.6215</v>
       </c>
       <c r="M8" t="n">
-        <v>-6</v>
+        <v>-3.76</v>
+      </c>
+      <c r="N8" t="n">
+        <v>9.859999999999999</v>
+      </c>
+      <c r="O8" t="n">
+        <v>6.31</v>
+      </c>
+      <c r="P8" t="n">
+        <v>1.5617</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>-3.17</v>
+      </c>
+      <c r="R8" t="n">
+        <v>14.96</v>
+      </c>
+      <c r="S8" t="n">
+        <v>12.04</v>
+      </c>
+      <c r="T8" t="n">
+        <v>1.2431</v>
+      </c>
+      <c r="U8" t="n">
+        <v>-7.42</v>
       </c>
     </row>
     <row r="9">
@@ -763,40 +939,64 @@
         <v>2005</v>
       </c>
       <c r="B9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" t="n">
+        <v>10.28</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.2918</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-7.17</v>
+      </c>
+      <c r="F9" t="n">
         <v>7.85</v>
       </c>
-      <c r="C9" t="n">
+      <c r="G9" t="n">
         <v>10.67</v>
       </c>
-      <c r="D9" t="n">
+      <c r="H9" t="n">
         <v>0.7354000000000001</v>
-      </c>
-      <c r="E9" t="n">
-        <v>-6.81</v>
-      </c>
-      <c r="F9" t="n">
-        <v>7.88</v>
-      </c>
-      <c r="G9" t="n">
-        <v>10.68</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0.7375</v>
       </c>
       <c r="I9" t="n">
         <v>-6.81</v>
       </c>
       <c r="J9" t="n">
-        <v>7.88</v>
+        <v>9.58</v>
       </c>
       <c r="K9" t="n">
-        <v>10.68</v>
+        <v>10.63</v>
       </c>
       <c r="L9" t="n">
-        <v>0.7375</v>
+        <v>0.9016999999999999</v>
       </c>
       <c r="M9" t="n">
-        <v>-6.81</v>
+        <v>-6.67</v>
+      </c>
+      <c r="N9" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="O9" t="n">
+        <v>8.01</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.6387</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>-4.93</v>
+      </c>
+      <c r="R9" t="n">
+        <v>29.33</v>
+      </c>
+      <c r="S9" t="n">
+        <v>18.67</v>
+      </c>
+      <c r="T9" t="n">
+        <v>1.5712</v>
+      </c>
+      <c r="U9" t="n">
+        <v>-13.35</v>
       </c>
     </row>
     <row r="10">
@@ -804,40 +1004,64 @@
         <v>2006</v>
       </c>
       <c r="B10" t="n">
+        <v>13.62</v>
+      </c>
+      <c r="C10" t="n">
+        <v>10.03</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1.3585</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-7.7</v>
+      </c>
+      <c r="F10" t="n">
         <v>16.28</v>
       </c>
-      <c r="C10" t="n">
+      <c r="G10" t="n">
         <v>10.22</v>
       </c>
-      <c r="D10" t="n">
+      <c r="H10" t="n">
         <v>1.5929</v>
       </c>
-      <c r="E10" t="n">
+      <c r="I10" t="n">
         <v>-7.57</v>
       </c>
-      <c r="F10" t="n">
-        <v>17.06</v>
-      </c>
-      <c r="G10" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="H10" t="n">
-        <v>1.4955</v>
-      </c>
-      <c r="I10" t="n">
-        <v>-8.390000000000001</v>
-      </c>
       <c r="J10" t="n">
-        <v>17.06</v>
+        <v>14.09</v>
       </c>
       <c r="K10" t="n">
-        <v>11.4</v>
+        <v>9.33</v>
       </c>
       <c r="L10" t="n">
-        <v>1.4955</v>
+        <v>1.5098</v>
       </c>
       <c r="M10" t="n">
-        <v>-8.390000000000001</v>
+        <v>-6.45</v>
+      </c>
+      <c r="N10" t="n">
+        <v>12.66</v>
+      </c>
+      <c r="O10" t="n">
+        <v>7.96</v>
+      </c>
+      <c r="P10" t="n">
+        <v>1.592</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>-5.4</v>
+      </c>
+      <c r="R10" t="n">
+        <v>19.28</v>
+      </c>
+      <c r="S10" t="n">
+        <v>20.27</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0.9513</v>
+      </c>
+      <c r="U10" t="n">
+        <v>-11.96</v>
       </c>
     </row>
     <row r="11">
@@ -845,16 +1069,16 @@
         <v>2007</v>
       </c>
       <c r="B11" t="n">
-        <v>9.66</v>
+        <v>3.53</v>
       </c>
       <c r="C11" t="n">
-        <v>15.47</v>
+        <v>15.99</v>
       </c>
       <c r="D11" t="n">
-        <v>0.6243</v>
+        <v>0.2208</v>
       </c>
       <c r="E11" t="n">
-        <v>-9.289999999999999</v>
+        <v>-10.09</v>
       </c>
       <c r="F11" t="n">
         <v>9.66</v>
@@ -869,16 +1093,40 @@
         <v>-9.289999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>9.66</v>
+        <v>8.77</v>
       </c>
       <c r="K11" t="n">
-        <v>15.47</v>
+        <v>13.93</v>
       </c>
       <c r="L11" t="n">
-        <v>0.6243</v>
+        <v>0.6297</v>
       </c>
       <c r="M11" t="n">
-        <v>-9.289999999999999</v>
+        <v>-8.390000000000001</v>
+      </c>
+      <c r="N11" t="n">
+        <v>5.96</v>
+      </c>
+      <c r="O11" t="n">
+        <v>12.42</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0.4803</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>-7.39</v>
+      </c>
+      <c r="R11" t="n">
+        <v>8.77</v>
+      </c>
+      <c r="S11" t="n">
+        <v>13.93</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0.6297</v>
+      </c>
+      <c r="U11" t="n">
+        <v>-8.390000000000001</v>
       </c>
     </row>
     <row r="12">
@@ -886,40 +1134,64 @@
         <v>2008</v>
       </c>
       <c r="B12" t="n">
+        <v>-38.49</v>
+      </c>
+      <c r="C12" t="n">
+        <v>40.97</v>
+      </c>
+      <c r="D12" t="n">
+        <v>-0.9393</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-48.01</v>
+      </c>
+      <c r="F12" t="n">
         <v>-34.26</v>
       </c>
-      <c r="C12" t="n">
+      <c r="G12" t="n">
         <v>38.25</v>
       </c>
-      <c r="D12" t="n">
+      <c r="H12" t="n">
         <v>-0.8956</v>
       </c>
-      <c r="E12" t="n">
+      <c r="I12" t="n">
         <v>-45.49</v>
       </c>
-      <c r="F12" t="n">
-        <v>-33.82</v>
-      </c>
-      <c r="G12" t="n">
-        <v>39.24</v>
-      </c>
-      <c r="H12" t="n">
-        <v>-0.8618</v>
-      </c>
-      <c r="I12" t="n">
-        <v>-45.29</v>
-      </c>
       <c r="J12" t="n">
-        <v>-33.82</v>
+        <v>-21.78</v>
       </c>
       <c r="K12" t="n">
-        <v>39.24</v>
+        <v>24.27</v>
       </c>
       <c r="L12" t="n">
-        <v>-0.8618</v>
+        <v>-0.8975</v>
       </c>
       <c r="M12" t="n">
-        <v>-45.29</v>
+        <v>-29.48</v>
+      </c>
+      <c r="N12" t="n">
+        <v>-20.34</v>
+      </c>
+      <c r="O12" t="n">
+        <v>22.07</v>
+      </c>
+      <c r="P12" t="n">
+        <v>-0.9216</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>-27.19</v>
+      </c>
+      <c r="R12" t="n">
+        <v>-39.48</v>
+      </c>
+      <c r="S12" t="n">
+        <v>57.12</v>
+      </c>
+      <c r="T12" t="n">
+        <v>-0.6912</v>
+      </c>
+      <c r="U12" t="n">
+        <v>-55.43</v>
       </c>
     </row>
     <row r="13">
@@ -927,40 +1199,64 @@
         <v>2009</v>
       </c>
       <c r="B13" t="n">
+        <v>23.45</v>
+      </c>
+      <c r="C13" t="n">
+        <v>27.29</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.8596</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-27.62</v>
+      </c>
+      <c r="F13" t="n">
         <v>29.28</v>
       </c>
-      <c r="C13" t="n">
+      <c r="G13" t="n">
         <v>27.25</v>
       </c>
-      <c r="D13" t="n">
+      <c r="H13" t="n">
         <v>1.0743</v>
       </c>
-      <c r="E13" t="n">
+      <c r="I13" t="n">
         <v>-27.68</v>
       </c>
-      <c r="F13" t="n">
-        <v>21.2</v>
-      </c>
-      <c r="G13" t="n">
-        <v>20.55</v>
-      </c>
-      <c r="H13" t="n">
-        <v>1.0319</v>
-      </c>
-      <c r="I13" t="n">
-        <v>-22.99</v>
-      </c>
       <c r="J13" t="n">
-        <v>20.2</v>
+        <v>2.59</v>
       </c>
       <c r="K13" t="n">
-        <v>19.4</v>
+        <v>3.03</v>
       </c>
       <c r="L13" t="n">
-        <v>1.0408</v>
+        <v>0.8556</v>
       </c>
       <c r="M13" t="n">
-        <v>-23.12</v>
+        <v>-3.8</v>
+      </c>
+      <c r="N13" t="n">
+        <v>7.04</v>
+      </c>
+      <c r="O13" t="n">
+        <v>7.19</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0.9791</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>-8.98</v>
+      </c>
+      <c r="R13" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="S13" t="n">
+        <v>4.89</v>
+      </c>
+      <c r="T13" t="n">
+        <v>0.8527</v>
+      </c>
+      <c r="U13" t="n">
+        <v>-6.09</v>
       </c>
     </row>
     <row r="14">
@@ -968,40 +1264,64 @@
         <v>2010</v>
       </c>
       <c r="B14" t="n">
+        <v>12.78</v>
+      </c>
+      <c r="C14" t="n">
+        <v>18.05</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.7081</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-15.99</v>
+      </c>
+      <c r="F14" t="n">
         <v>16.09</v>
       </c>
-      <c r="C14" t="n">
+      <c r="G14" t="n">
         <v>18.06</v>
       </c>
-      <c r="D14" t="n">
+      <c r="H14" t="n">
         <v>0.8911</v>
       </c>
-      <c r="E14" t="n">
+      <c r="I14" t="n">
         <v>-15.19</v>
       </c>
-      <c r="F14" t="n">
-        <v>18.48</v>
-      </c>
-      <c r="G14" t="n">
-        <v>20.96</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0.8819</v>
-      </c>
-      <c r="I14" t="n">
-        <v>-18.1</v>
-      </c>
       <c r="J14" t="n">
-        <v>18.45</v>
+        <v>6.6</v>
       </c>
       <c r="K14" t="n">
-        <v>19.93</v>
+        <v>7.47</v>
       </c>
       <c r="L14" t="n">
-        <v>0.9256</v>
+        <v>0.8832</v>
       </c>
       <c r="M14" t="n">
-        <v>-17.33</v>
+        <v>-6.5</v>
+      </c>
+      <c r="N14" t="n">
+        <v>4.73</v>
+      </c>
+      <c r="O14" t="n">
+        <v>7.11</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0.6657</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>-5.24</v>
+      </c>
+      <c r="R14" t="n">
+        <v>17.92</v>
+      </c>
+      <c r="S14" t="n">
+        <v>20.86</v>
+      </c>
+      <c r="T14" t="n">
+        <v>0.859</v>
+      </c>
+      <c r="U14" t="n">
+        <v>-17.94</v>
       </c>
     </row>
     <row r="15">
@@ -1009,40 +1329,64 @@
         <v>2011</v>
       </c>
       <c r="B15" t="n">
+        <v>-0</v>
+      </c>
+      <c r="C15" t="n">
+        <v>23.27</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-0.0001</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-19.39</v>
+      </c>
+      <c r="F15" t="n">
         <v>3.11</v>
       </c>
-      <c r="C15" t="n">
+      <c r="G15" t="n">
         <v>23.07</v>
       </c>
-      <c r="D15" t="n">
+      <c r="H15" t="n">
         <v>0.1347</v>
       </c>
-      <c r="E15" t="n">
+      <c r="I15" t="n">
         <v>-18.61</v>
       </c>
-      <c r="F15" t="n">
-        <v>3.09</v>
-      </c>
-      <c r="G15" t="n">
-        <v>23.08</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0.1341</v>
-      </c>
-      <c r="I15" t="n">
-        <v>-18.62</v>
-      </c>
       <c r="J15" t="n">
-        <v>3.09</v>
+        <v>7.76</v>
       </c>
       <c r="K15" t="n">
-        <v>23.08</v>
+        <v>12.59</v>
       </c>
       <c r="L15" t="n">
-        <v>0.1341</v>
+        <v>0.6167</v>
       </c>
       <c r="M15" t="n">
-        <v>-18.62</v>
+        <v>-9.699999999999999</v>
+      </c>
+      <c r="N15" t="n">
+        <v>7.68</v>
+      </c>
+      <c r="O15" t="n">
+        <v>12.58</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0.6104000000000001</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>-9.76</v>
+      </c>
+      <c r="R15" t="n">
+        <v>-0.36</v>
+      </c>
+      <c r="S15" t="n">
+        <v>26.84</v>
+      </c>
+      <c r="T15" t="n">
+        <v>-0.0135</v>
+      </c>
+      <c r="U15" t="n">
+        <v>-24.33</v>
       </c>
     </row>
     <row r="16">
@@ -1050,40 +1394,64 @@
         <v>2012</v>
       </c>
       <c r="B16" t="n">
+        <v>13.41</v>
+      </c>
+      <c r="C16" t="n">
+        <v>12.77</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-9.94</v>
+      </c>
+      <c r="F16" t="n">
         <v>14.66</v>
       </c>
-      <c r="C16" t="n">
+      <c r="G16" t="n">
         <v>12.22</v>
       </c>
-      <c r="D16" t="n">
+      <c r="H16" t="n">
         <v>1.1998</v>
       </c>
-      <c r="E16" t="n">
+      <c r="I16" t="n">
         <v>-8.789999999999999</v>
       </c>
-      <c r="F16" t="n">
-        <v>11.58</v>
-      </c>
-      <c r="G16" t="n">
-        <v>10.35</v>
-      </c>
-      <c r="H16" t="n">
-        <v>1.1186</v>
-      </c>
-      <c r="I16" t="n">
-        <v>-7.05</v>
-      </c>
       <c r="J16" t="n">
-        <v>11.58</v>
+        <v>6.28</v>
       </c>
       <c r="K16" t="n">
-        <v>10.35</v>
+        <v>5.38</v>
       </c>
       <c r="L16" t="n">
-        <v>1.1186</v>
+        <v>1.1688</v>
       </c>
       <c r="M16" t="n">
-        <v>-7.05</v>
+        <v>-4.3</v>
+      </c>
+      <c r="N16" t="n">
+        <v>6.81</v>
+      </c>
+      <c r="O16" t="n">
+        <v>5.54</v>
+      </c>
+      <c r="P16" t="n">
+        <v>1.2298</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>-4.29</v>
+      </c>
+      <c r="R16" t="n">
+        <v>9.369999999999999</v>
+      </c>
+      <c r="S16" t="n">
+        <v>9.039999999999999</v>
+      </c>
+      <c r="T16" t="n">
+        <v>1.0366</v>
+      </c>
+      <c r="U16" t="n">
+        <v>-7.17</v>
       </c>
     </row>
     <row r="17">
@@ -1091,40 +1459,64 @@
         <v>2013</v>
       </c>
       <c r="B17" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="C17" t="n">
+        <v>11.07</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2.6743</v>
+      </c>
+      <c r="E17" t="n">
+        <v>-5.76</v>
+      </c>
+      <c r="F17" t="n">
         <v>30.86</v>
-      </c>
-      <c r="C17" t="n">
-        <v>11.03</v>
-      </c>
-      <c r="D17" t="n">
-        <v>2.7978</v>
-      </c>
-      <c r="E17" t="n">
-        <v>-5.94</v>
-      </c>
-      <c r="F17" t="n">
-        <v>30.88</v>
       </c>
       <c r="G17" t="n">
         <v>11.03</v>
       </c>
       <c r="H17" t="n">
-        <v>2.7989</v>
+        <v>2.7978</v>
       </c>
       <c r="I17" t="n">
         <v>-5.94</v>
       </c>
       <c r="J17" t="n">
-        <v>30.88</v>
+        <v>25.68</v>
       </c>
       <c r="K17" t="n">
-        <v>11.03</v>
+        <v>9.32</v>
       </c>
       <c r="L17" t="n">
-        <v>2.7989</v>
+        <v>2.7561</v>
       </c>
       <c r="M17" t="n">
-        <v>-5.94</v>
+        <v>-5.11</v>
+      </c>
+      <c r="N17" t="n">
+        <v>23.64</v>
+      </c>
+      <c r="O17" t="n">
+        <v>8.52</v>
+      </c>
+      <c r="P17" t="n">
+        <v>2.7758</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>-4.69</v>
+      </c>
+      <c r="R17" t="n">
+        <v>35.79</v>
+      </c>
+      <c r="S17" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="T17" t="n">
+        <v>3.0372</v>
+      </c>
+      <c r="U17" t="n">
+        <v>-5.52</v>
       </c>
     </row>
     <row r="18">
@@ -1132,16 +1524,16 @@
         <v>2014</v>
       </c>
       <c r="B18" t="n">
-        <v>13.33</v>
+        <v>11.39</v>
       </c>
       <c r="C18" t="n">
-        <v>10.98</v>
+        <v>11.37</v>
       </c>
       <c r="D18" t="n">
-        <v>1.2145</v>
+        <v>1.0018</v>
       </c>
       <c r="E18" t="n">
-        <v>-7.05</v>
+        <v>-7.4</v>
       </c>
       <c r="F18" t="n">
         <v>13.33</v>
@@ -1150,22 +1542,46 @@
         <v>10.98</v>
       </c>
       <c r="H18" t="n">
-        <v>1.2137</v>
+        <v>1.2145</v>
       </c>
       <c r="I18" t="n">
         <v>-7.05</v>
       </c>
       <c r="J18" t="n">
-        <v>13.33</v>
+        <v>13.87</v>
       </c>
       <c r="K18" t="n">
-        <v>10.98</v>
+        <v>10.53</v>
       </c>
       <c r="L18" t="n">
-        <v>1.2137</v>
+        <v>1.3174</v>
       </c>
       <c r="M18" t="n">
-        <v>-7.05</v>
+        <v>-6.27</v>
+      </c>
+      <c r="N18" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="O18" t="n">
+        <v>8.92</v>
+      </c>
+      <c r="P18" t="n">
+        <v>1.2783</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>-5.59</v>
+      </c>
+      <c r="R18" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="S18" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="T18" t="n">
+        <v>1.0607</v>
+      </c>
+      <c r="U18" t="n">
+        <v>-7.72</v>
       </c>
     </row>
     <row r="19">
@@ -1173,40 +1589,64 @@
         <v>2015</v>
       </c>
       <c r="B19" t="n">
+        <v>-0.73</v>
+      </c>
+      <c r="C19" t="n">
+        <v>15.49</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-0.0469</v>
+      </c>
+      <c r="E19" t="n">
+        <v>-12.35</v>
+      </c>
+      <c r="F19" t="n">
         <v>-1.34</v>
       </c>
-      <c r="C19" t="n">
+      <c r="G19" t="n">
         <v>15.1</v>
       </c>
-      <c r="D19" t="n">
+      <c r="H19" t="n">
         <v>-0.08890000000000001</v>
       </c>
-      <c r="E19" t="n">
+      <c r="I19" t="n">
         <v>-12.55</v>
       </c>
-      <c r="F19" t="n">
-        <v>1.59</v>
-      </c>
-      <c r="G19" t="n">
-        <v>14.52</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0.1098</v>
-      </c>
-      <c r="I19" t="n">
-        <v>-10.27</v>
-      </c>
       <c r="J19" t="n">
-        <v>1.59</v>
+        <v>1.77</v>
       </c>
       <c r="K19" t="n">
-        <v>14.52</v>
+        <v>14.01</v>
       </c>
       <c r="L19" t="n">
-        <v>0.1098</v>
+        <v>0.1267</v>
       </c>
       <c r="M19" t="n">
-        <v>-10.27</v>
+        <v>-9.58</v>
+      </c>
+      <c r="N19" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="O19" t="n">
+        <v>11.96</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0.1345</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>-8.550000000000001</v>
+      </c>
+      <c r="R19" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="S19" t="n">
+        <v>14.47</v>
+      </c>
+      <c r="T19" t="n">
+        <v>0.131</v>
+      </c>
+      <c r="U19" t="n">
+        <v>-9.880000000000001</v>
       </c>
     </row>
     <row r="20">
@@ -1214,40 +1654,64 @@
         <v>2016</v>
       </c>
       <c r="B20" t="n">
+        <v>9.539999999999999</v>
+      </c>
+      <c r="C20" t="n">
+        <v>13.09</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.7281</v>
+      </c>
+      <c r="E20" t="n">
+        <v>-9.300000000000001</v>
+      </c>
+      <c r="F20" t="n">
         <v>14.37</v>
       </c>
-      <c r="C20" t="n">
+      <c r="G20" t="n">
         <v>12.81</v>
       </c>
-      <c r="D20" t="n">
+      <c r="H20" t="n">
         <v>1.1217</v>
       </c>
-      <c r="E20" t="n">
+      <c r="I20" t="n">
         <v>-7.91</v>
       </c>
-      <c r="F20" t="n">
-        <v>10.86</v>
-      </c>
-      <c r="G20" t="n">
-        <v>12.09</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0.8984</v>
-      </c>
-      <c r="I20" t="n">
-        <v>-7.7</v>
-      </c>
       <c r="J20" t="n">
-        <v>10.86</v>
+        <v>4.26</v>
       </c>
       <c r="K20" t="n">
-        <v>12.09</v>
+        <v>7.98</v>
       </c>
       <c r="L20" t="n">
-        <v>0.8984</v>
+        <v>0.5345</v>
       </c>
       <c r="M20" t="n">
-        <v>-7.7</v>
+        <v>-4.68</v>
+      </c>
+      <c r="N20" t="n">
+        <v>7.79</v>
+      </c>
+      <c r="O20" t="n">
+        <v>7.58</v>
+      </c>
+      <c r="P20" t="n">
+        <v>1.0275</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>-4.36</v>
+      </c>
+      <c r="R20" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="S20" t="n">
+        <v>10.87</v>
+      </c>
+      <c r="T20" t="n">
+        <v>0.9002</v>
+      </c>
+      <c r="U20" t="n">
+        <v>-6.94</v>
       </c>
     </row>
     <row r="21">
@@ -1255,40 +1719,64 @@
         <v>2017</v>
       </c>
       <c r="B21" t="n">
+        <v>19.42</v>
+      </c>
+      <c r="C21" t="n">
+        <v>6.69</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2.9047</v>
+      </c>
+      <c r="E21" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="F21" t="n">
         <v>19.22</v>
       </c>
-      <c r="C21" t="n">
+      <c r="G21" t="n">
         <v>6.28</v>
       </c>
-      <c r="D21" t="n">
+      <c r="H21" t="n">
         <v>3.0596</v>
       </c>
-      <c r="E21" t="n">
+      <c r="I21" t="n">
         <v>-2.57</v>
       </c>
-      <c r="F21" t="n">
-        <v>16.78</v>
-      </c>
-      <c r="G21" t="n">
-        <v>7.55</v>
-      </c>
-      <c r="H21" t="n">
-        <v>2.2223</v>
-      </c>
-      <c r="I21" t="n">
-        <v>-3.87</v>
-      </c>
       <c r="J21" t="n">
-        <v>16.78</v>
+        <v>15.97</v>
       </c>
       <c r="K21" t="n">
-        <v>7.55</v>
+        <v>4.92</v>
       </c>
       <c r="L21" t="n">
-        <v>2.2223</v>
+        <v>3.2451</v>
       </c>
       <c r="M21" t="n">
-        <v>-3.87</v>
+        <v>-1.76</v>
+      </c>
+      <c r="N21" t="n">
+        <v>15.33</v>
+      </c>
+      <c r="O21" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="P21" t="n">
+        <v>3.4588</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>-1.45</v>
+      </c>
+      <c r="R21" t="n">
+        <v>16.24</v>
+      </c>
+      <c r="S21" t="n">
+        <v>7.76</v>
+      </c>
+      <c r="T21" t="n">
+        <v>2.0939</v>
+      </c>
+      <c r="U21" t="n">
+        <v>-4.14</v>
       </c>
     </row>
     <row r="22">
@@ -1296,40 +1784,64 @@
         <v>2018</v>
       </c>
       <c r="B22" t="n">
+        <v>-6.24</v>
+      </c>
+      <c r="C22" t="n">
+        <v>17.05</v>
+      </c>
+      <c r="D22" t="n">
+        <v>-0.3658</v>
+      </c>
+      <c r="E22" t="n">
+        <v>-19.78</v>
+      </c>
+      <c r="F22" t="n">
         <v>-6.17</v>
       </c>
-      <c r="C22" t="n">
+      <c r="G22" t="n">
         <v>15.35</v>
       </c>
-      <c r="D22" t="n">
+      <c r="H22" t="n">
         <v>-0.4017</v>
-      </c>
-      <c r="E22" t="n">
-        <v>-18.47</v>
-      </c>
-      <c r="F22" t="n">
-        <v>-6.16</v>
-      </c>
-      <c r="G22" t="n">
-        <v>15.36</v>
-      </c>
-      <c r="H22" t="n">
-        <v>-0.4011</v>
       </c>
       <c r="I22" t="n">
         <v>-18.47</v>
       </c>
       <c r="J22" t="n">
-        <v>-6.16</v>
+        <v>-5.05</v>
       </c>
       <c r="K22" t="n">
-        <v>15.36</v>
+        <v>16.39</v>
       </c>
       <c r="L22" t="n">
-        <v>-0.4011</v>
+        <v>-0.3082</v>
       </c>
       <c r="M22" t="n">
-        <v>-18.47</v>
+        <v>-18.86</v>
+      </c>
+      <c r="N22" t="n">
+        <v>-5.05</v>
+      </c>
+      <c r="O22" t="n">
+        <v>16.39</v>
+      </c>
+      <c r="P22" t="n">
+        <v>-0.3082</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>-18.86</v>
+      </c>
+      <c r="R22" t="n">
+        <v>-5.05</v>
+      </c>
+      <c r="S22" t="n">
+        <v>16.39</v>
+      </c>
+      <c r="T22" t="n">
+        <v>-0.3082</v>
+      </c>
+      <c r="U22" t="n">
+        <v>-18.86</v>
       </c>
     </row>
     <row r="23">
@@ -1337,40 +1849,64 @@
         <v>2019</v>
       </c>
       <c r="B23" t="n">
+        <v>28.88</v>
+      </c>
+      <c r="C23" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="D23" t="n">
+        <v>2.3154</v>
+      </c>
+      <c r="E23" t="n">
+        <v>-6.84</v>
+      </c>
+      <c r="F23" t="n">
         <v>27.89</v>
       </c>
-      <c r="C23" t="n">
+      <c r="G23" t="n">
         <v>11.58</v>
       </c>
-      <c r="D23" t="n">
+      <c r="H23" t="n">
         <v>2.4094</v>
       </c>
-      <c r="E23" t="n">
+      <c r="I23" t="n">
         <v>-6.35</v>
       </c>
-      <c r="F23" t="n">
-        <v>30.03</v>
-      </c>
-      <c r="G23" t="n">
-        <v>10.75</v>
-      </c>
-      <c r="H23" t="n">
-        <v>2.7935</v>
-      </c>
-      <c r="I23" t="n">
-        <v>-5.05</v>
-      </c>
       <c r="J23" t="n">
-        <v>30.03</v>
+        <v>21.72</v>
       </c>
       <c r="K23" t="n">
-        <v>10.75</v>
+        <v>7.46</v>
       </c>
       <c r="L23" t="n">
-        <v>2.7935</v>
+        <v>2.9125</v>
       </c>
       <c r="M23" t="n">
-        <v>-5.05</v>
+        <v>-3.42</v>
+      </c>
+      <c r="N23" t="n">
+        <v>15.27</v>
+      </c>
+      <c r="O23" t="n">
+        <v>5.82</v>
+      </c>
+      <c r="P23" t="n">
+        <v>2.623</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>-2.68</v>
+      </c>
+      <c r="R23" t="n">
+        <v>24.87</v>
+      </c>
+      <c r="S23" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="T23" t="n">
+        <v>2.7046</v>
+      </c>
+      <c r="U23" t="n">
+        <v>-4.29</v>
       </c>
     </row>
     <row r="24">
@@ -1378,40 +1914,64 @@
         <v>2020</v>
       </c>
       <c r="B24" t="n">
+        <v>16.26</v>
+      </c>
+      <c r="C24" t="n">
+        <v>34.43</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.4722</v>
+      </c>
+      <c r="E24" t="n">
+        <v>-33.92</v>
+      </c>
+      <c r="F24" t="n">
         <v>10.37</v>
       </c>
-      <c r="C24" t="n">
+      <c r="G24" t="n">
         <v>35.62</v>
       </c>
-      <c r="D24" t="n">
+      <c r="H24" t="n">
         <v>0.2912</v>
       </c>
-      <c r="E24" t="n">
+      <c r="I24" t="n">
         <v>-36.91</v>
       </c>
-      <c r="F24" t="n">
-        <v>10.41</v>
-      </c>
-      <c r="G24" t="n">
-        <v>35.61</v>
-      </c>
-      <c r="H24" t="n">
-        <v>0.2924</v>
-      </c>
-      <c r="I24" t="n">
-        <v>-36.9</v>
-      </c>
       <c r="J24" t="n">
-        <v>10.41</v>
+        <v>9.81</v>
       </c>
       <c r="K24" t="n">
-        <v>35.61</v>
+        <v>31.28</v>
       </c>
       <c r="L24" t="n">
-        <v>0.2924</v>
+        <v>0.3135</v>
       </c>
       <c r="M24" t="n">
-        <v>-36.9</v>
+        <v>-32.98</v>
+      </c>
+      <c r="N24" t="n">
+        <v>12.86</v>
+      </c>
+      <c r="O24" t="n">
+        <v>25.89</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0.4969</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>-26.83</v>
+      </c>
+      <c r="R24" t="n">
+        <v>43.62</v>
+      </c>
+      <c r="S24" t="n">
+        <v>40.17</v>
+      </c>
+      <c r="T24" t="n">
+        <v>1.086</v>
+      </c>
+      <c r="U24" t="n">
+        <v>-31.15</v>
       </c>
     </row>
     <row r="25">
@@ -1419,40 +1979,64 @@
         <v>2021</v>
       </c>
       <c r="B25" t="n">
+        <v>26.89</v>
+      </c>
+      <c r="C25" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>2.0529</v>
+      </c>
+      <c r="E25" t="n">
+        <v>-5.21</v>
+      </c>
+      <c r="F25" t="n">
         <v>29.6</v>
       </c>
-      <c r="C25" t="n">
+      <c r="G25" t="n">
         <v>12.55</v>
       </c>
-      <c r="D25" t="n">
+      <c r="H25" t="n">
         <v>2.3582</v>
       </c>
-      <c r="E25" t="n">
+      <c r="I25" t="n">
         <v>-4.69</v>
       </c>
-      <c r="F25" t="n">
-        <v>28.43</v>
-      </c>
-      <c r="G25" t="n">
-        <v>13.58</v>
-      </c>
-      <c r="H25" t="n">
-        <v>2.0935</v>
-      </c>
-      <c r="I25" t="n">
-        <v>-5.33</v>
-      </c>
       <c r="J25" t="n">
-        <v>28.21</v>
+        <v>7.64</v>
       </c>
       <c r="K25" t="n">
-        <v>13.43</v>
+        <v>3.58</v>
       </c>
       <c r="L25" t="n">
-        <v>2.0995</v>
+        <v>2.1334</v>
       </c>
       <c r="M25" t="n">
-        <v>-5.41</v>
+        <v>-2.02</v>
+      </c>
+      <c r="N25" t="n">
+        <v>9.85</v>
+      </c>
+      <c r="O25" t="n">
+        <v>5.39</v>
+      </c>
+      <c r="P25" t="n">
+        <v>1.8287</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>-2.82</v>
+      </c>
+      <c r="R25" t="n">
+        <v>32.04</v>
+      </c>
+      <c r="S25" t="n">
+        <v>16.54</v>
+      </c>
+      <c r="T25" t="n">
+        <v>1.9366</v>
+      </c>
+      <c r="U25" t="n">
+        <v>-7.39</v>
       </c>
     </row>
     <row r="26">
@@ -1460,40 +2044,64 @@
         <v>2022</v>
       </c>
       <c r="B26" t="n">
+        <v>-19.44</v>
+      </c>
+      <c r="C26" t="n">
+        <v>24.17</v>
+      </c>
+      <c r="D26" t="n">
+        <v>-0.8043</v>
+      </c>
+      <c r="E26" t="n">
+        <v>-25.43</v>
+      </c>
+      <c r="F26" t="n">
         <v>-5.15</v>
       </c>
-      <c r="C26" t="n">
+      <c r="G26" t="n">
         <v>21.08</v>
       </c>
-      <c r="D26" t="n">
+      <c r="H26" t="n">
         <v>-0.2445</v>
       </c>
-      <c r="E26" t="n">
+      <c r="I26" t="n">
         <v>-16.94</v>
       </c>
-      <c r="F26" t="n">
-        <v>-2.73</v>
-      </c>
-      <c r="G26" t="n">
-        <v>24.51</v>
-      </c>
-      <c r="H26" t="n">
-        <v>-0.1116</v>
-      </c>
-      <c r="I26" t="n">
-        <v>-18.31</v>
-      </c>
       <c r="J26" t="n">
-        <v>-2.73</v>
+        <v>-5.28</v>
       </c>
       <c r="K26" t="n">
-        <v>24.51</v>
+        <v>17.48</v>
       </c>
       <c r="L26" t="n">
-        <v>-0.1116</v>
+        <v>-0.3023</v>
       </c>
       <c r="M26" t="n">
-        <v>-18.31</v>
+        <v>-14.26</v>
+      </c>
+      <c r="N26" t="n">
+        <v>-5.39</v>
+      </c>
+      <c r="O26" t="n">
+        <v>13.84</v>
+      </c>
+      <c r="P26" t="n">
+        <v>-0.3897</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>-12.35</v>
+      </c>
+      <c r="R26" t="n">
+        <v>64.08</v>
+      </c>
+      <c r="S26" t="n">
+        <v>35.23</v>
+      </c>
+      <c r="T26" t="n">
+        <v>1.819</v>
+      </c>
+      <c r="U26" t="n">
+        <v>-26.01</v>
       </c>
     </row>
     <row r="27">
@@ -1501,40 +2109,64 @@
         <v>2023</v>
       </c>
       <c r="B27" t="n">
+        <v>24.23</v>
+      </c>
+      <c r="C27" t="n">
+        <v>13.09</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1.8507</v>
+      </c>
+      <c r="E27" t="n">
+        <v>-10.28</v>
+      </c>
+      <c r="F27" t="n">
         <v>13.89</v>
       </c>
-      <c r="C27" t="n">
+      <c r="G27" t="n">
         <v>12.24</v>
       </c>
-      <c r="D27" t="n">
+      <c r="H27" t="n">
         <v>1.1352</v>
       </c>
-      <c r="E27" t="n">
+      <c r="I27" t="n">
         <v>-10.11</v>
       </c>
-      <c r="F27" t="n">
-        <v>3.77</v>
-      </c>
-      <c r="G27" t="n">
-        <v>12.51</v>
-      </c>
-      <c r="H27" t="n">
-        <v>0.3014</v>
-      </c>
-      <c r="I27" t="n">
-        <v>-8.960000000000001</v>
-      </c>
       <c r="J27" t="n">
-        <v>3.77</v>
+        <v>0.32</v>
       </c>
       <c r="K27" t="n">
-        <v>12.51</v>
+        <v>6.48</v>
       </c>
       <c r="L27" t="n">
-        <v>0.3014</v>
+        <v>0.049</v>
       </c>
       <c r="M27" t="n">
-        <v>-8.960000000000001</v>
+        <v>-5.04</v>
+      </c>
+      <c r="N27" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="O27" t="n">
+        <v>6.62</v>
+      </c>
+      <c r="P27" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>-5.24</v>
+      </c>
+      <c r="R27" t="n">
+        <v>-0.63</v>
+      </c>
+      <c r="S27" t="n">
+        <v>22.91</v>
+      </c>
+      <c r="T27" t="n">
+        <v>-0.0275</v>
+      </c>
+      <c r="U27" t="n">
+        <v>-17.33</v>
       </c>
     </row>
     <row r="28">
@@ -1542,47 +2174,73 @@
         <v>2024</v>
       </c>
       <c r="B28" t="n">
+        <v>23.84</v>
+      </c>
+      <c r="C28" t="n">
+        <v>12.66</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1.8824</v>
+      </c>
+      <c r="E28" t="n">
+        <v>-8.49</v>
+      </c>
+      <c r="F28" t="n">
         <v>15.76</v>
       </c>
-      <c r="C28" t="n">
+      <c r="G28" t="n">
         <v>10.39</v>
       </c>
-      <c r="D28" t="n">
+      <c r="H28" t="n">
         <v>1.5166</v>
       </c>
-      <c r="E28" t="n">
+      <c r="I28" t="n">
         <v>-6.47</v>
       </c>
-      <c r="F28" t="n">
-        <v>19.35</v>
-      </c>
-      <c r="G28" t="n">
-        <v>13.53</v>
-      </c>
-      <c r="H28" t="n">
-        <v>1.4303</v>
-      </c>
-      <c r="I28" t="n">
-        <v>-9.300000000000001</v>
-      </c>
       <c r="J28" t="n">
-        <v>19.35</v>
+        <v>12.93</v>
       </c>
       <c r="K28" t="n">
-        <v>13.53</v>
+        <v>8.51</v>
       </c>
       <c r="L28" t="n">
-        <v>1.4303</v>
+        <v>1.5196</v>
       </c>
       <c r="M28" t="n">
-        <v>-9.300000000000001</v>
+        <v>-5.46</v>
+      </c>
+      <c r="N28" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="O28" t="n">
+        <v>10.23</v>
+      </c>
+      <c r="P28" t="n">
+        <v>1.2699</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>-7.53</v>
+      </c>
+      <c r="R28" t="n">
+        <v>24.85</v>
+      </c>
+      <c r="S28" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="T28" t="n">
+        <v>1.2808</v>
+      </c>
+      <c r="U28" t="n">
+        <v>-14.77</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="J1:M1"/>
+  <mergeCells count="5">
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="F1:I1"/>
+    <mergeCell ref="R1:U1"/>
+    <mergeCell ref="N1:Q1"/>
+    <mergeCell ref="J1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>